<commit_message>
Enable submit workflow for job applications
</commit_message>
<xml_diff>
--- a/JOB_APPLICATION_TRACKER.xlsx
+++ b/JOB_APPLICATION_TRACKER.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R673935d5713245ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI" sheetId="2" r:id="Rbd8f127f655249b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SDE" sheetId="3" r:id="Rdf594e15dbfa4c38"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blockers" sheetId="4" r:id="R81951a45fb554c8f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R33f59c14501d466e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI" sheetId="2" r:id="Rd794b5deebde4751"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SDE" sheetId="3" r:id="Rfe7396da8ab54e0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blockers" sheetId="4" r:id="R95b57114298f4c72"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -364,17 +364,17 @@
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
       <x:c r="A10" s="2" t="str">
-        <x:v>AI roles prepared</x:v>
-      </x:c>
-      <x:c r="B10" s="2" t="n">
-        <x:v>0</x:v>
+        <x:v>Daily target</x:v>
+      </x:c>
+      <x:c r="B10" s="2" t="str">
+        <x:v>Up to 100 real-fit applications when enough matching roles are available</x:v>
       </x:c>
       <x:c r="C10" s="2"/>
       <x:c r="D10" s="2"/>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="2" t="str">
-        <x:v>SDE roles prepared</x:v>
+        <x:v>Applications submitted</x:v>
       </x:c>
       <x:c r="B11" s="2" t="n">
         <x:v>0</x:v>
@@ -384,7 +384,7 @@
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
       <x:c r="A12" s="2" t="str">
-        <x:v>Gmail drafts created</x:v>
+        <x:v>Gmail confirmations found</x:v>
       </x:c>
       <x:c r="B12" s="2" t="n">
         <x:v>0</x:v>
@@ -394,13 +394,27 @@
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
       <x:c r="A13" s="2" t="str">
-        <x:v>Applications submitted by Vineesha</x:v>
+        <x:v>Gmail drafts created</x:v>
       </x:c>
       <x:c r="B13" s="2" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="C13" s="2"/>
       <x:c r="D13" s="2"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:v>Blocked for review</x:v>
+      </x:c>
+      <x:c r="B14" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="str">
+        <x:v>Last run notes</x:v>
+      </x:c>
+      <x:c r="B15" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -453,7 +467,7 @@
         <x:v>Work Authorization</x:v>
       </x:c>
       <x:c r="J1" s="5" t="str">
-        <x:v>Draft Link / Notes</x:v>
+        <x:v>Confirmation / Draft / Notes</x:v>
       </x:c>
       <x:c r="K1" s="5" t="str">
         <x:v>Next Action</x:v>
@@ -510,7 +524,7 @@
         <x:v>Work Authorization</x:v>
       </x:c>
       <x:c r="J1" s="5" t="str">
-        <x:v>Draft Link / Notes</x:v>
+        <x:v>Confirmation / Draft / Notes</x:v>
       </x:c>
       <x:c r="K1" s="5" t="str">
         <x:v>Next Action</x:v>

</xml_diff>